<commit_message>
bug fixed with full app developed
</commit_message>
<xml_diff>
--- a/assets/sample/sample_file.xlsx
+++ b/assets/sample/sample_file.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parth\StudioProjects\quiz_battle\assets\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28BFF110-54C3-4D7F-A494-C77484E7EBB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{501B288E-4DBB-4841-A529-646A830195A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{F6C96A48-85C7-45F5-9A7A-EB5CCF06E874}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="58">
   <si>
     <t>Question</t>
   </si>
@@ -87,6 +87,129 @@
   </si>
   <si>
     <t>Microsoft</t>
+  </si>
+  <si>
+    <t>What is the capital of India?</t>
+  </si>
+  <si>
+    <t>Mumbai</t>
+  </si>
+  <si>
+    <t>Delhi</t>
+  </si>
+  <si>
+    <t>Chennai</t>
+  </si>
+  <si>
+    <t>Kolkata</t>
+  </si>
+  <si>
+    <t>Which planet is known as the Red Planet?</t>
+  </si>
+  <si>
+    <t>Earth</t>
+  </si>
+  <si>
+    <t>Venus</t>
+  </si>
+  <si>
+    <t>Mars</t>
+  </si>
+  <si>
+    <t>Jupiter</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>Who is known as the Father of Computers?</t>
+  </si>
+  <si>
+    <t>Charles Babbage</t>
+  </si>
+  <si>
+    <t>Albert Einstein</t>
+  </si>
+  <si>
+    <t>Isaac Newton</t>
+  </si>
+  <si>
+    <t>Alan Turing</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>What is the largest ocean on Earth?</t>
+  </si>
+  <si>
+    <t>Atlantic Ocean</t>
+  </si>
+  <si>
+    <t>Indian Ocean</t>
+  </si>
+  <si>
+    <t>Pacific Ocean</t>
+  </si>
+  <si>
+    <t>Arctic Ocean</t>
+  </si>
+  <si>
+    <t>Which programming language is used in Flutter?</t>
+  </si>
+  <si>
+    <t>Java</t>
+  </si>
+  <si>
+    <t>Kotlin</t>
+  </si>
+  <si>
+    <t>Dart</t>
+  </si>
+  <si>
+    <t>Python</t>
+  </si>
+  <si>
+    <t>How many continents are there in the world?</t>
+  </si>
+  <si>
+    <t>What is the national animal of India?</t>
+  </si>
+  <si>
+    <t>Lion</t>
+  </si>
+  <si>
+    <t>Tiger</t>
+  </si>
+  <si>
+    <t>Elephant</t>
+  </si>
+  <si>
+    <t>Peacock</t>
+  </si>
+  <si>
+    <t>Which gas do plants absorb from the atmosphere?</t>
+  </si>
+  <si>
+    <t>Oxygen</t>
+  </si>
+  <si>
+    <t>Nitrogen</t>
+  </si>
+  <si>
+    <t>Carbon Dioxide</t>
+  </si>
+  <si>
+    <t>Hydrogen</t>
+  </si>
+  <si>
+    <t>What is the value of π (Pi) approximately?</t>
+  </si>
+  <si>
+    <t>Which company developed Flutter?</t>
+  </si>
+  <si>
+    <t>D</t>
   </si>
 </sst>
 </file>
@@ -130,9 +253,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -467,7 +593,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18EAF004-45AA-414A-B042-D735C6916478}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -534,6 +660,206 @@
         <v>11</v>
       </c>
     </row>
+    <row r="4" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="2">
+        <v>5</v>
+      </c>
+      <c r="C9" s="2">
+        <v>6</v>
+      </c>
+      <c r="D9" s="2">
+        <v>7</v>
+      </c>
+      <c r="E9" s="2">
+        <v>8</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B12" s="2">
+        <v>2.14</v>
+      </c>
+      <c r="C12" s="2">
+        <v>3.14</v>
+      </c>
+      <c r="D12" s="2">
+        <v>4.1399999999999997</v>
+      </c>
+      <c r="E12" s="2">
+        <v>5.14</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Solve Edit Profile conflicts
</commit_message>
<xml_diff>
--- a/assets/sample/sample_file.xlsx
+++ b/assets/sample/sample_file.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\parth\StudioProjects\quiz_battle\assets\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{501B288E-4DBB-4841-A529-646A830195A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B389D72F-F2B0-4A1C-AD72-6E4F68181E5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{F6C96A48-85C7-45F5-9A7A-EB5CCF06E874}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{F6C96A48-85C7-45F5-9A7A-EB5CCF06E874}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="161">
   <si>
     <t>Question</t>
   </si>
@@ -210,6 +210,315 @@
   </si>
   <si>
     <t>D</t>
+  </si>
+  <si>
+    <t>What does CPU stand for?</t>
+  </si>
+  <si>
+    <t>Central Process Unit</t>
+  </si>
+  <si>
+    <t>Central Processing Unit</t>
+  </si>
+  <si>
+    <t>Computer Processing Unit</t>
+  </si>
+  <si>
+    <t>Control Processing Unit</t>
+  </si>
+  <si>
+    <t>Which language is primarily used for Android app development?</t>
+  </si>
+  <si>
+    <t>Swift</t>
+  </si>
+  <si>
+    <t>C#</t>
+  </si>
+  <si>
+    <t>What is the capital of Gujarat?</t>
+  </si>
+  <si>
+    <t>Surat</t>
+  </si>
+  <si>
+    <t>Rajkot</t>
+  </si>
+  <si>
+    <t>Ahmedabad</t>
+  </si>
+  <si>
+    <t>Gandhinagar</t>
+  </si>
+  <si>
+    <t>Which planet is the largest in the Solar System?</t>
+  </si>
+  <si>
+    <t>Saturn</t>
+  </si>
+  <si>
+    <t>Neptune</t>
+  </si>
+  <si>
+    <t>What is the national flower of India?</t>
+  </si>
+  <si>
+    <t>Lotus</t>
+  </si>
+  <si>
+    <t>Rose</t>
+  </si>
+  <si>
+    <t>Sunflower</t>
+  </si>
+  <si>
+    <t>Lily</t>
+  </si>
+  <si>
+    <t>Which data structure follows the FIFO principle?</t>
+  </si>
+  <si>
+    <t>Stack</t>
+  </si>
+  <si>
+    <t>Queue</t>
+  </si>
+  <si>
+    <t>Tree</t>
+  </si>
+  <si>
+    <t>Graph</t>
+  </si>
+  <si>
+    <t>What is the full form of HTML?</t>
+  </si>
+  <si>
+    <t>Hyper Text Markup Language</t>
+  </si>
+  <si>
+    <t>High Text Machine Language</t>
+  </si>
+  <si>
+    <t>Hyper Tool Markup Language</t>
+  </si>
+  <si>
+    <t>Home Text Markup Language</t>
+  </si>
+  <si>
+    <t>Which widget is used to create a scrollable list in Flutter?</t>
+  </si>
+  <si>
+    <t>Column</t>
+  </si>
+  <si>
+    <t>Container</t>
+  </si>
+  <si>
+    <t>ListView</t>
+  </si>
+  <si>
+    <t>Row</t>
+  </si>
+  <si>
+    <t>Which country is known as the Land of the Rising Sun?</t>
+  </si>
+  <si>
+    <t>China</t>
+  </si>
+  <si>
+    <t>Thailand</t>
+  </si>
+  <si>
+    <t>Japan</t>
+  </si>
+  <si>
+    <t>South Korea</t>
+  </si>
+  <si>
+    <t>What is the chemical symbol for Water?</t>
+  </si>
+  <si>
+    <t>HO</t>
+  </si>
+  <si>
+    <t>H2O</t>
+  </si>
+  <si>
+    <t>HO2</t>
+  </si>
+  <si>
+    <t>H3O</t>
+  </si>
+  <si>
+    <t>Which is the smallest prime number?</t>
+  </si>
+  <si>
+    <t>What is the default file extension for Dart files?</t>
+  </si>
+  <si>
+    <t>.java</t>
+  </si>
+  <si>
+    <t>.dart</t>
+  </si>
+  <si>
+    <t>.flutter</t>
+  </si>
+  <si>
+    <t>.kt</t>
+  </si>
+  <si>
+    <t>Which keyword is used to declare a constant in Dart?</t>
+  </si>
+  <si>
+    <t>final</t>
+  </si>
+  <si>
+    <t>var</t>
+  </si>
+  <si>
+    <t>const</t>
+  </si>
+  <si>
+    <t>static</t>
+  </si>
+  <si>
+    <t>Which device is used to input text into a computer?</t>
+  </si>
+  <si>
+    <t>Monitor</t>
+  </si>
+  <si>
+    <t>Printer</t>
+  </si>
+  <si>
+    <t>Keyboard</t>
+  </si>
+  <si>
+    <t>Speaker</t>
+  </si>
+  <si>
+    <t>What does URL stand for?</t>
+  </si>
+  <si>
+    <t>Uniform Resource Locator</t>
+  </si>
+  <si>
+    <t>Universal Resource Link</t>
+  </si>
+  <si>
+    <t>Unified Resource Locator</t>
+  </si>
+  <si>
+    <t>Uniform Reference Link</t>
+  </si>
+  <si>
+    <t>Which widget is commonly used for button clicks in Flutter?</t>
+  </si>
+  <si>
+    <t>Scaffold</t>
+  </si>
+  <si>
+    <t>AppBar</t>
+  </si>
+  <si>
+    <t>ElevatedButton</t>
+  </si>
+  <si>
+    <t>Text</t>
+  </si>
+  <si>
+    <t>What is the national sport of India (commonly recognized)?</t>
+  </si>
+  <si>
+    <t>Cricket</t>
+  </si>
+  <si>
+    <t>Hockey</t>
+  </si>
+  <si>
+    <t>Football</t>
+  </si>
+  <si>
+    <t>Kabaddi</t>
+  </si>
+  <si>
+    <t>Which planet is closest to the Sun?</t>
+  </si>
+  <si>
+    <t>Mercury</t>
+  </si>
+  <si>
+    <t>What is the largest mammal in the world?</t>
+  </si>
+  <si>
+    <t>Blue Whale</t>
+  </si>
+  <si>
+    <t>Giraffe</t>
+  </si>
+  <si>
+    <t>Hippopotamus</t>
+  </si>
+  <si>
+    <t>Which company developed the Android operating system?</t>
+  </si>
+  <si>
+    <t>IBM</t>
+  </si>
+  <si>
+    <t>What does RAM stand for?</t>
+  </si>
+  <si>
+    <t>Random Access Memory</t>
+  </si>
+  <si>
+    <t>Read Access Memory</t>
+  </si>
+  <si>
+    <t>Rapid Access Memory</t>
+  </si>
+  <si>
+    <t>Real Access Memory</t>
+  </si>
+  <si>
+    <t>Which widget is used as the root of a Flutter app?</t>
+  </si>
+  <si>
+    <t>MaterialApp</t>
+  </si>
+  <si>
+    <t>How many states are there in India?</t>
+  </si>
+  <si>
+    <t>Which programming language is used for web page styling?</t>
+  </si>
+  <si>
+    <t>HTML</t>
+  </si>
+  <si>
+    <t>CSS</t>
+  </si>
+  <si>
+    <t>JavaScript</t>
+  </si>
+  <si>
+    <t>SQL</t>
+  </si>
+  <si>
+    <t>What is the currency of India?</t>
+  </si>
+  <si>
+    <t>Dollar</t>
+  </si>
+  <si>
+    <t>Euro</t>
+  </si>
+  <si>
+    <t>Yen</t>
+  </si>
+  <si>
+    <t>Rupee</t>
   </si>
 </sst>
 </file>
@@ -593,7 +902,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18EAF004-45AA-414A-B042-D735C6916478}">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -860,6 +1169,506 @@
         <v>57</v>
       </c>
     </row>
+    <row r="14" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A17" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A19" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A21" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A22" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A23" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B24" s="2">
+        <v>0</v>
+      </c>
+      <c r="C24" s="2">
+        <v>1</v>
+      </c>
+      <c r="D24" s="2">
+        <v>2</v>
+      </c>
+      <c r="E24" s="2">
+        <v>3</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A25" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A29" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A30" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A31" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A32" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A33" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B36" s="2">
+        <v>26</v>
+      </c>
+      <c r="C36" s="2">
+        <v>27</v>
+      </c>
+      <c r="D36" s="2">
+        <v>28</v>
+      </c>
+      <c r="E36" s="2">
+        <v>29</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A38" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>